<commit_message>
Mudanças na estrutura de continentes
</commit_message>
<xml_diff>
--- a/core/src/main/resources/baseFiles/excel/Sheet.xlsx
+++ b/core/src/main/resources/baseFiles/excel/Sheet.xlsx
@@ -1216,34 +1216,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
antes de uma grande mudança
</commit_message>
<xml_diff>
--- a/core/src/main/resources/baseFiles/excel/Sheet.xlsx
+++ b/core/src/main/resources/baseFiles/excel/Sheet.xlsx
@@ -1216,34 +1216,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
More firms and before structural changes
</commit_message>
<xml_diff>
--- a/core/src/main/resources/baseFiles/excel/Sheet.xlsx
+++ b/core/src/main/resources/baseFiles/excel/Sheet.xlsx
@@ -1216,34 +1216,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" t="s" s="0">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" t="s" s="0">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" t="s" s="0">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" t="s" s="0">
         <v>9</v>
       </c>
     </row>

</xml_diff>